<commit_message>
Add playoff prediction summary to matches
</commit_message>
<xml_diff>
--- a/server/uploads/predictions/Ennustus_avo.xlsx
+++ b/server/uploads/predictions/Ennustus_avo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AvoOk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\luupinite-ennustus-2026\server\uploads\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE157EB-1495-40C5-8A11-A57F8656F2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CAD196-8584-4AAC-9F82-16D2549255EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="1455" windowWidth="21600" windowHeight="11295" xr2:uid="{71ACDA5A-2A4F-42DF-A035-BA793F8CA08E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{71ACDA5A-2A4F-42DF-A035-BA793F8CA08E}"/>
   </bookViews>
   <sheets>
     <sheet name="Ennustus" sheetId="1" r:id="rId1"/>
@@ -1585,7 +1585,7 @@
         <v>79</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Lisasin playoffi ennustused nähtavaks
</commit_message>
<xml_diff>
--- a/server/uploads/predictions/Ennustus_avo.xlsx
+++ b/server/uploads/predictions/Ennustus_avo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AvoOk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\luupinite-ennustus-2026\server\uploads\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE157EB-1495-40C5-8A11-A57F8656F2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E93F7C-4D4E-4B3A-A526-90AA77F7A567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="1455" windowWidth="21600" windowHeight="11295" xr2:uid="{71ACDA5A-2A4F-42DF-A035-BA793F8CA08E}"/>
+    <workbookView xWindow="7995" yWindow="3705" windowWidth="21600" windowHeight="11235" xr2:uid="{71ACDA5A-2A4F-42DF-A035-BA793F8CA08E}"/>
   </bookViews>
   <sheets>
     <sheet name="Ennustus" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="97">
   <si>
     <t>Kodus</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t>Kanada</t>
+  </si>
+  <si>
+    <t>prantsusmaa</t>
   </si>
 </sst>
 </file>
@@ -1611,7 +1614,7 @@
         <v>90</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">

</xml_diff>